<commit_message>
chore: actualizar Excel de outcomes
</commit_message>
<xml_diff>
--- a/docs/Breakoutbot_Outcomes.xlsx
+++ b/docs/Breakoutbot_Outcomes.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1320,6 +1320,1862 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:50</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="D14" t="n">
+        <v>70</v>
+      </c>
+      <c r="E14" t="n">
+        <v>257.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>-23.75</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UFG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:50</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1715</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1075.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.6264999999999999</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>-31.72</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PRHI</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:50</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="D16" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" t="n">
+        <v>214.11</v>
+      </c>
+      <c r="F16" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7.5528</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GRI</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:50</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2.4045</v>
+      </c>
+      <c r="D17" t="n">
+        <v>161</v>
+      </c>
+      <c r="E17" t="n">
+        <v>387.12</v>
+      </c>
+      <c r="F17" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>76.56999999999999</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ELOX</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:50</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>16.47</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>115.29</v>
+      </c>
+      <c r="F18" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G18" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H18" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="I18" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="J18" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>-15.68</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BSEM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:52</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3.775</v>
+      </c>
+      <c r="D19" t="n">
+        <v>64</v>
+      </c>
+      <c r="E19" t="n">
+        <v>241.6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3.699</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>YQ</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:56</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="D20" t="n">
+        <v>232</v>
+      </c>
+      <c r="E20" t="n">
+        <v>628.72</v>
+      </c>
+      <c r="F20" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.6583</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-4</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:57</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1.3401</v>
+      </c>
+      <c r="D21" t="n">
+        <v>80</v>
+      </c>
+      <c r="E21" t="n">
+        <v>107.21</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J21" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>-13.02</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NRSN</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:03</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="D22" t="n">
+        <v>260</v>
+      </c>
+      <c r="E22" t="n">
+        <v>115.7</v>
+      </c>
+      <c r="F22" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.4105</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J22" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>-16.64</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SPWR</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:06</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.3706</v>
+      </c>
+      <c r="D23" t="n">
+        <v>434</v>
+      </c>
+      <c r="E23" t="n">
+        <v>160.84</v>
+      </c>
+      <c r="F23" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.3655</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.3437</v>
+      </c>
+      <c r="J23" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>-12.85</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NDRA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:06</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="D24" t="n">
+        <v>33</v>
+      </c>
+      <c r="E24" t="n">
+        <v>199.65</v>
+      </c>
+      <c r="F24" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="H24" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ZOOZ</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:25</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>8.1999</v>
+      </c>
+      <c r="D25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E25" t="n">
+        <v>262.4</v>
+      </c>
+      <c r="F25" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="H25" t="n">
+        <v>8.265000000000001</v>
+      </c>
+      <c r="I25" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>-12.81</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TREO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:25</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="D26" t="n">
+        <v>167</v>
+      </c>
+      <c r="E26" t="n">
+        <v>855.04</v>
+      </c>
+      <c r="F26" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="J26" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>-20.01</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EJH</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:25</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1.2617</v>
+      </c>
+      <c r="D27" t="n">
+        <v>115</v>
+      </c>
+      <c r="E27" t="n">
+        <v>145.1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:25</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D28" t="n">
+        <v>11</v>
+      </c>
+      <c r="E28" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="F28" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G28" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="I28" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J28" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ZTG</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:36</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.7302999999999999</v>
+      </c>
+      <c r="D29" t="n">
+        <v>115</v>
+      </c>
+      <c r="E29" t="n">
+        <v>83.98</v>
+      </c>
+      <c r="F29" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.7299</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J29" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="P29" s="3" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GMHS</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:36</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.8567</v>
+      </c>
+      <c r="D30" t="n">
+        <v>188</v>
+      </c>
+      <c r="E30" t="n">
+        <v>161.06</v>
+      </c>
+      <c r="F30" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.8199</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="J30" t="n">
+        <v>9</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>-10.42</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:40</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="D31" t="n">
+        <v>8</v>
+      </c>
+      <c r="E31" t="n">
+        <v>99.36</v>
+      </c>
+      <c r="F31" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G31" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="H31" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="I31" t="n">
+        <v>11</v>
+      </c>
+      <c r="J31" t="n">
+        <v>-13.1</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="M31" s="3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="P31" s="3" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MIRA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:47</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0.7739</v>
+      </c>
+      <c r="D32" t="n">
+        <v>692</v>
+      </c>
+      <c r="E32" t="n">
+        <v>535.54</v>
+      </c>
+      <c r="F32" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.7571</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.7571</v>
+      </c>
+      <c r="J32" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>-7.02</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FBGL</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:51</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="D33" t="n">
+        <v>295</v>
+      </c>
+      <c r="E33" t="n">
+        <v>117.7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.3597</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.3597</v>
+      </c>
+      <c r="J33" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>-6.54</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:04</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>4.855</v>
+      </c>
+      <c r="D34" t="n">
+        <v>24</v>
+      </c>
+      <c r="E34" t="n">
+        <v>116.52</v>
+      </c>
+      <c r="F34" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="G34" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="H34" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="I34" t="n">
+        <v>4.385</v>
+      </c>
+      <c r="J34" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>-2.28</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NTRB</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:45</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>5.6699</v>
+      </c>
+      <c r="D35" t="n">
+        <v>30</v>
+      </c>
+      <c r="E35" t="n">
+        <v>170.1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="H35" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="I35" t="n">
+        <v>5.304</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="L35" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M35" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="P35" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:45</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3.4947</v>
+      </c>
+      <c r="D36" t="n">
+        <v>61</v>
+      </c>
+      <c r="E36" t="n">
+        <v>213.18</v>
+      </c>
+      <c r="F36" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="G36" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3.489</v>
+      </c>
+      <c r="I36" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NWGL</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:53</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1.1363</v>
+      </c>
+      <c r="D37" t="n">
+        <v>69</v>
+      </c>
+      <c r="E37" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="F37" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1.265</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="J37" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="L37" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="M37" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="N37" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MBRX</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:59</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0.7371</v>
+      </c>
+      <c r="D38" t="n">
+        <v>195</v>
+      </c>
+      <c r="E38" t="n">
+        <v>143.73</v>
+      </c>
+      <c r="F38" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.6949</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J38" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>FLZH</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-04 12:03</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="D39" t="n">
+        <v>953</v>
+      </c>
+      <c r="E39" t="n">
+        <v>84.81999999999999</v>
+      </c>
+      <c r="F39" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.07729999999999999</v>
+      </c>
+      <c r="J39" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>-8.48</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BTCS</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-09-04 12:40</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="D40" t="n">
+        <v>278</v>
+      </c>
+      <c r="E40" t="n">
+        <v>400.32</v>
+      </c>
+      <c r="F40" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.519</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-4</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DUO</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-09-04 13:40</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0.5789</v>
+      </c>
+      <c r="D41" t="n">
+        <v>286</v>
+      </c>
+      <c r="E41" t="n">
+        <v>165.57</v>
+      </c>
+      <c r="F41" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.5566</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J41" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AEHL</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-09-04 13:44</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7</v>
+      </c>
+      <c r="E42" t="n">
+        <v>58.03</v>
+      </c>
+      <c r="F42" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="G42" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="H42" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="I42" t="n">
+        <v>6.7665</v>
+      </c>
+      <c r="J42" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>-0.84</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1355,7 +3211,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2401.8</v>
+        <v>2307.86</v>
       </c>
     </row>
     <row r="3">
@@ -1365,7 +3221,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-98.2</v>
+        <v>-192.14</v>
       </c>
     </row>
     <row r="4">
@@ -1375,7 +3231,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-3.93</v>
+        <v>-7.69</v>
       </c>
     </row>
     <row r="5">
@@ -1385,7 +3241,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -1395,7 +3251,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -1405,7 +3261,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>